<commit_message>
Update automation/runner.py to generate 350 real test cases per workbook during CI/CD execution
</commit_message>
<xml_diff>
--- a/automation/Automation_Test_Report.xlsx
+++ b/automation/Automation_Test_Report.xlsx
@@ -526,7 +526,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G34"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
     <col width="50" customWidth="1" min="2" max="2"/>
@@ -1199,7 +1199,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:J351"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
     <col width="49" customWidth="1" min="2" max="2"/>

</xml_diff>